<commit_message>
Add housing fair HTML assets and update source data
</commit_message>
<xml_diff>
--- a/src/topics.xlsx
+++ b/src/topics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sakoda.kouhei\Documents\GitHub\corporate-partnership-portal-20260309141849\src\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1E2DF04-ADE0-4D15-BECE-CF88773123D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F84FE81-C8CA-46F1-A1CE-B7C105F16D07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-19310" yWindow="-80" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="シート1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="25">
   <si>
     <t>予定</t>
   </si>
@@ -46,28 +46,16 @@
     <t>ＰＲ活動</t>
   </si>
   <si>
-    <t>ベルス　タカラレーベン・レーベンホームビルド🏠資料請求キャンペーン公開中✨</t>
-  </si>
-  <si>
     <t>1</t>
   </si>
   <si>
     <t>新規契約</t>
   </si>
   <si>
-    <t>新規提携企業：東京都医師協同組合連合会　との提携を開始しました</t>
-  </si>
-  <si>
     <t>来場誘致</t>
   </si>
   <si>
     <t>ベルス主催の住宅フェア参加　職域企業36社参加</t>
-  </si>
-  <si>
-    <t>新規提携企業：パナソニック共済会　との提携を開始しました</t>
-  </si>
-  <si>
-    <t>新規提携企業：東京海上日動ファシリティーズ　との提携を開始しました</t>
   </si>
   <si>
     <t>「株式会社リロクラブ」日本最大：福利厚生倶楽部</t>
@@ -101,6 +89,134 @@
     </rPh>
     <phoneticPr fontId="2"/>
   </si>
+  <si>
+    <t>来場誘致</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>新規契約</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>東京都医師協同組合連合会　との提携を開始しました</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>パナソニック共済会　との提携を開始しました</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>東京海上日動ファシリティーズ　との提携を開始しました</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>三菱電機ライフサービスとの新規提携を開始しました</t>
+    <rPh sb="0" eb="2">
+      <t>ミツビシ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>デンキ</t>
+    </rPh>
+    <rPh sb="13" eb="15">
+      <t>シンキ</t>
+    </rPh>
+    <rPh sb="15" eb="17">
+      <t>テイケイ</t>
+    </rPh>
+    <rPh sb="18" eb="20">
+      <t>カイシ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>SBアットワーク（ソフトバンク）との新規提携を開始しました</t>
+    <rPh sb="18" eb="20">
+      <t>シンキ</t>
+    </rPh>
+    <rPh sb="20" eb="22">
+      <t>テイケイ</t>
+    </rPh>
+    <rPh sb="23" eb="25">
+      <t>カイシ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>コーサイ・サービス（防衛省）との新規提携を開始しました</t>
+    <rPh sb="10" eb="13">
+      <t>ボウエイショウ</t>
+    </rPh>
+    <rPh sb="16" eb="18">
+      <t>シンキ</t>
+    </rPh>
+    <rPh sb="18" eb="20">
+      <t>テイケイ</t>
+    </rPh>
+    <rPh sb="21" eb="23">
+      <t>カイシ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="3"/>
+      </rPr>
+      <t>✨</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="HGPｺﾞｼｯｸM"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>ベルス主催の住宅相談フェア参加</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Segoe UI Symbol"/>
+        <family val="3"/>
+      </rPr>
+      <t>🏠</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="HGPｺﾞｼｯｸM"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>　詳細はコチラclick</t>
+    </r>
+    <rPh sb="4" eb="6">
+      <t>シュサイ</t>
+    </rPh>
+    <rPh sb="7" eb="9">
+      <t>ジュウタク</t>
+    </rPh>
+    <rPh sb="9" eb="11">
+      <t>ソウダン</t>
+    </rPh>
+    <rPh sb="14" eb="16">
+      <t>サンカ</t>
+    </rPh>
+    <rPh sb="19" eb="21">
+      <t>ショウサイ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>ベルス　タカラレーベン・レーベンホームビルド資料請求キャンペーン公開中</t>
+    <phoneticPr fontId="2"/>
+  </si>
 </sst>
 </file>
 
@@ -109,7 +225,7 @@
   <numFmts count="1">
     <numFmt numFmtId="176" formatCode="yyyy/mm/dd"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -152,6 +268,12 @@
       <family val="1"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Segoe UI Symbol"/>
+      <family val="3"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -173,7 +295,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="176" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -185,6 +307,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -331,7 +456,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="HOJIN_TOPIC_お知らせ更新情報" displayName="HOJIN_TOPIC_お知らせ更新情報" ref="A1:C8" headerRowDxfId="5" dataDxfId="4" totalsRowDxfId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="HOJIN_TOPIC_お知らせ更新情報" displayName="HOJIN_TOPIC_お知らせ更新情報" ref="A1:C12" headerRowDxfId="5" dataDxfId="4" totalsRowDxfId="3">
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="予定" dataDxfId="2"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="目的" dataDxfId="1"/>
@@ -542,8 +667,8 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
-  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <dimension ref="A1:H12"/>
+  <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
@@ -557,7 +682,7 @@
     <col min="11" max="11" width="11.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="22.5" customHeight="1">
+    <row r="1" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -571,7 +696,7 @@
         <v>3</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F1" t="s">
         <v>4</v>
@@ -583,129 +708,175 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="22.5" customHeight="1">
-      <c r="A2" s="1">
+    <row r="2" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="5">
+        <v>46101</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E2" s="4"/>
+    </row>
+    <row r="3" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="5">
+        <v>46106</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" s="4"/>
+    </row>
+    <row r="4" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="5">
+        <v>46106</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" s="4"/>
+    </row>
+    <row r="5" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="5">
+        <v>46099</v>
+      </c>
+      <c r="B5" s="1"/>
+      <c r="C5" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" s="4"/>
+    </row>
+    <row r="6" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="1">
         <v>46054</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B6" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C6" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" t="s">
         <v>8</v>
-      </c>
-      <c r="E2" t="s">
-        <v>9</v>
-      </c>
-      <c r="H2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="22.5" customHeight="1">
-      <c r="A3" s="1">
-        <v>46052</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" t="s">
-        <v>9</v>
-      </c>
-      <c r="H3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="22.5" customHeight="1">
-      <c r="A4" s="1">
-        <v>46051</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E4" t="s">
-        <v>9</v>
-      </c>
-      <c r="H4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="22.5" customHeight="1">
-      <c r="A5" s="1">
-        <v>46045</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D5" t="s">
-        <v>9</v>
-      </c>
-      <c r="H5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="22.5" customHeight="1">
-      <c r="A6" s="1">
-        <v>46045</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D6" t="s">
-        <v>9</v>
       </c>
       <c r="H6">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="22.5" customHeight="1">
+    <row r="7" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
-        <v>46003</v>
+        <v>46052</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D7" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H7">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="22.5" customHeight="1">
+    <row r="8" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
+        <v>46051</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
+        <v>8</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="1">
+        <v>46045</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" t="s">
+        <v>8</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="1">
+        <v>46045</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10" t="s">
+        <v>8</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="1">
+        <v>46003</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D11" t="s">
+        <v>8</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="1">
         <v>45992</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B12" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E8" t="s">
-        <v>9</v>
-      </c>
-      <c r="H8">
+      <c r="C12" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E12" t="s">
+        <v>8</v>
+      </c>
+      <c r="H12">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2"/>
   <dataValidations count="1">
-    <dataValidation type="list" sqref="D2:H200" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" sqref="D6:H204" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"1,0"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>